<commit_message>
Update scenario_defaults.xlsx to reflect new data configurations
</commit_message>
<xml_diff>
--- a/database/scenario_defaults.xlsx
+++ b/database/scenario_defaults.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cypri\OneDrive\Documents\1. Pro\Formations\Jupyter Notebooks\pyPPA\French_PPA\database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9426f84fd314fc67/Documents/1. Pro/Formations/Jupyter Notebooks/French_PPA/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{34ABFB4C-B909-4BAD-BD6D-1709B4BFF71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{34ABFB4C-B909-4BAD-BD6D-1709B4BFF71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43DBAE20-39E1-4EAB-B87A-4809EC57D6A9}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19095" windowHeight="12075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="303">
   <si>
     <t>FRENCH PPA MODEL — scenario_defaults.xlsx</t>
   </si>
@@ -1164,20 +1164,20 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
@@ -1487,21 +1487,21 @@
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="55" customWidth="1"/>
+    <col min="9" max="9" width="58.53125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
     </row>
     <row r="2" spans="1:9" ht="50" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
@@ -1533,17 +1533,17 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="18"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="20"/>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
@@ -1574,7 +1574,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:9" ht="31.9" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>20</v>
       </c>
@@ -1604,17 +1604,17 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="18"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="20"/>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
@@ -1791,17 +1791,17 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="18"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="20"/>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
@@ -1862,17 +1862,17 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="18"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="20"/>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
@@ -1962,17 +1962,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="18"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
@@ -2091,17 +2091,17 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="17"/>
-      <c r="I25" s="18"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="20"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
@@ -2194,8 +2194,8 @@
       <c r="A29" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>37</v>
+      <c r="B29" s="4">
+        <v>5</v>
       </c>
       <c r="C29" s="4">
         <v>5</v>
@@ -2307,17 +2307,17 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="18"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="20"/>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
@@ -2523,17 +2523,17 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="16" t="s">
+      <c r="A41" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="18"/>
+      <c r="B41" s="19"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="20"/>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
@@ -2768,17 +2768,17 @@
       </c>
     </row>
     <row r="50" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="16" t="s">
+      <c r="A50" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B50" s="17"/>
-      <c r="C50" s="17"/>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="17"/>
-      <c r="G50" s="17"/>
-      <c r="H50" s="17"/>
-      <c r="I50" s="18"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="20"/>
     </row>
     <row r="51" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
@@ -2984,30 +2984,30 @@
       </c>
     </row>
     <row r="58" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="16" t="s">
+      <c r="A58" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B58" s="17"/>
-      <c r="C58" s="17"/>
-      <c r="D58" s="17"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="17"/>
-      <c r="G58" s="17"/>
-      <c r="H58" s="17"/>
-      <c r="I58" s="18"/>
+      <c r="B58" s="19"/>
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="19"/>
+      <c r="I58" s="20"/>
     </row>
     <row r="59" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" s="19" t="s">
+      <c r="A59" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="17"/>
-      <c r="I59" s="18"/>
+      <c r="B59" s="19"/>
+      <c r="C59" s="19"/>
+      <c r="D59" s="19"/>
+      <c r="E59" s="19"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="19"/>
+      <c r="I59" s="20"/>
     </row>
     <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
@@ -3068,30 +3068,30 @@
       </c>
     </row>
     <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A62" s="20" t="s">
+      <c r="A62" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="B62" s="17"/>
-      <c r="C62" s="17"/>
-      <c r="D62" s="17"/>
-      <c r="E62" s="17"/>
-      <c r="F62" s="17"/>
-      <c r="G62" s="17"/>
-      <c r="H62" s="17"/>
-      <c r="I62" s="18"/>
+      <c r="B62" s="19"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="19"/>
+      <c r="G62" s="19"/>
+      <c r="H62" s="19"/>
+      <c r="I62" s="20"/>
     </row>
     <row r="63" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A63" s="19" t="s">
+      <c r="A63" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="17"/>
-      <c r="D63" s="17"/>
-      <c r="E63" s="17"/>
-      <c r="F63" s="17"/>
-      <c r="G63" s="17"/>
-      <c r="H63" s="17"/>
-      <c r="I63" s="18"/>
+      <c r="B63" s="19"/>
+      <c r="C63" s="19"/>
+      <c r="D63" s="19"/>
+      <c r="E63" s="19"/>
+      <c r="F63" s="19"/>
+      <c r="G63" s="19"/>
+      <c r="H63" s="19"/>
+      <c r="I63" s="20"/>
     </row>
     <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
@@ -3152,17 +3152,17 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="19" t="s">
+      <c r="A66" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="17"/>
-      <c r="C66" s="17"/>
-      <c r="D66" s="17"/>
-      <c r="E66" s="17"/>
-      <c r="F66" s="17"/>
-      <c r="G66" s="17"/>
-      <c r="H66" s="17"/>
-      <c r="I66" s="18"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="19"/>
+      <c r="E66" s="19"/>
+      <c r="F66" s="19"/>
+      <c r="G66" s="19"/>
+      <c r="H66" s="19"/>
+      <c r="I66" s="20"/>
     </row>
     <row r="67" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
@@ -3252,17 +3252,17 @@
       </c>
     </row>
     <row r="70" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A70" s="19" t="s">
+      <c r="A70" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B70" s="17"/>
-      <c r="C70" s="17"/>
-      <c r="D70" s="17"/>
-      <c r="E70" s="17"/>
-      <c r="F70" s="17"/>
-      <c r="G70" s="17"/>
-      <c r="H70" s="17"/>
-      <c r="I70" s="18"/>
+      <c r="B70" s="19"/>
+      <c r="C70" s="19"/>
+      <c r="D70" s="19"/>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="19"/>
+      <c r="I70" s="20"/>
     </row>
     <row r="71" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="3" t="s">
@@ -3352,17 +3352,17 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A74" s="19" t="s">
+      <c r="A74" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="B74" s="17"/>
-      <c r="C74" s="17"/>
-      <c r="D74" s="17"/>
-      <c r="E74" s="17"/>
-      <c r="F74" s="17"/>
-      <c r="G74" s="17"/>
-      <c r="H74" s="17"/>
-      <c r="I74" s="18"/>
+      <c r="B74" s="19"/>
+      <c r="C74" s="19"/>
+      <c r="D74" s="19"/>
+      <c r="E74" s="19"/>
+      <c r="F74" s="19"/>
+      <c r="G74" s="19"/>
+      <c r="H74" s="19"/>
+      <c r="I74" s="20"/>
     </row>
     <row r="75" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="3" t="s">
@@ -3452,30 +3452,30 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" s="16" t="s">
+      <c r="A78" s="21" t="s">
         <v>183</v>
       </c>
-      <c r="B78" s="21"/>
-      <c r="C78" s="21"/>
-      <c r="D78" s="21"/>
-      <c r="E78" s="21"/>
-      <c r="F78" s="21"/>
-      <c r="G78" s="21"/>
-      <c r="H78" s="21"/>
-      <c r="I78" s="21"/>
+      <c r="B78" s="17"/>
+      <c r="C78" s="17"/>
+      <c r="D78" s="17"/>
+      <c r="E78" s="17"/>
+      <c r="F78" s="17"/>
+      <c r="G78" s="17"/>
+      <c r="H78" s="17"/>
+      <c r="I78" s="17"/>
     </row>
     <row r="79" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="19" t="s">
+      <c r="A79" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="B79" s="21"/>
-      <c r="C79" s="21"/>
-      <c r="D79" s="21"/>
-      <c r="E79" s="21"/>
-      <c r="F79" s="21"/>
-      <c r="G79" s="21"/>
-      <c r="H79" s="21"/>
-      <c r="I79" s="21"/>
+      <c r="B79" s="17"/>
+      <c r="C79" s="17"/>
+      <c r="D79" s="17"/>
+      <c r="E79" s="17"/>
+      <c r="F79" s="17"/>
+      <c r="G79" s="17"/>
+      <c r="H79" s="17"/>
+      <c r="I79" s="17"/>
     </row>
     <row r="80" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="13" t="s">
@@ -3681,17 +3681,17 @@
       </c>
     </row>
     <row r="87" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" s="19" t="s">
+      <c r="A87" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="B87" s="21"/>
-      <c r="C87" s="21"/>
-      <c r="D87" s="21"/>
-      <c r="E87" s="21"/>
-      <c r="F87" s="21"/>
-      <c r="G87" s="21"/>
-      <c r="H87" s="21"/>
-      <c r="I87" s="21"/>
+      <c r="B87" s="17"/>
+      <c r="C87" s="17"/>
+      <c r="D87" s="17"/>
+      <c r="E87" s="17"/>
+      <c r="F87" s="17"/>
+      <c r="G87" s="17"/>
+      <c r="H87" s="17"/>
+      <c r="I87" s="17"/>
     </row>
     <row r="88" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A88" s="13" t="s">
@@ -3868,17 +3868,17 @@
       </c>
     </row>
     <row r="94" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A94" s="19" t="s">
+      <c r="A94" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="B94" s="21"/>
-      <c r="C94" s="21"/>
-      <c r="D94" s="21"/>
-      <c r="E94" s="21"/>
-      <c r="F94" s="21"/>
-      <c r="G94" s="21"/>
-      <c r="H94" s="21"/>
-      <c r="I94" s="21"/>
+      <c r="B94" s="17"/>
+      <c r="C94" s="17"/>
+      <c r="D94" s="17"/>
+      <c r="E94" s="17"/>
+      <c r="F94" s="17"/>
+      <c r="G94" s="17"/>
+      <c r="H94" s="17"/>
+      <c r="I94" s="17"/>
     </row>
     <row r="95" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A95" s="13" t="s">
@@ -4026,17 +4026,17 @@
       </c>
     </row>
     <row r="100" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A100" s="19" t="s">
+      <c r="A100" s="18" t="s">
         <v>234</v>
       </c>
-      <c r="B100" s="21"/>
-      <c r="C100" s="21"/>
-      <c r="D100" s="21"/>
-      <c r="E100" s="21"/>
-      <c r="F100" s="21"/>
-      <c r="G100" s="21"/>
-      <c r="H100" s="21"/>
-      <c r="I100" s="21"/>
+      <c r="B100" s="17"/>
+      <c r="C100" s="17"/>
+      <c r="D100" s="17"/>
+      <c r="E100" s="17"/>
+      <c r="F100" s="17"/>
+      <c r="G100" s="17"/>
+      <c r="H100" s="17"/>
+      <c r="I100" s="17"/>
     </row>
     <row r="101" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="3" t="s">
@@ -4325,7 +4325,7 @@
       <c r="H111" s="11"/>
       <c r="I111" s="12"/>
     </row>
-    <row r="112" spans="1:9" ht="23.25" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:9" ht="34.9" x14ac:dyDescent="0.45">
       <c r="A112" s="3" t="s">
         <v>262</v>
       </c>
@@ -4443,6 +4443,19 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A100:I100"/>
+    <mergeCell ref="A63:I63"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A58:I58"/>
+    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A66:I66"/>
+    <mergeCell ref="A74:I74"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="A62:I62"/>
+    <mergeCell ref="A20:I20"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A94:I94"/>
     <mergeCell ref="A70:I70"/>
@@ -4451,20 +4464,7 @@
     <mergeCell ref="A87:I87"/>
     <mergeCell ref="A78:I78"/>
     <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A100:I100"/>
-    <mergeCell ref="A63:I63"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A58:I58"/>
-    <mergeCell ref="A59:I59"/>
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A66:I66"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A74:I74"/>
-    <mergeCell ref="A50:I50"/>
-    <mergeCell ref="A33:I33"/>
-    <mergeCell ref="A62:I62"/>
-    <mergeCell ref="A20:I20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4483,9 +4483,9 @@
       <c r="A1" s="23" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="7"/>

</xml_diff>

<commit_message>
Update scenario_defaults.xlsx to incorporate updated data configurations
</commit_message>
<xml_diff>
--- a/database/scenario_defaults.xlsx
+++ b/database/scenario_defaults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9426f84fd314fc67/Documents/1. Pro/Formations/Jupyter Notebooks/French_PPA/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{34ABFB4C-B909-4BAD-BD6D-1709B4BFF71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43DBAE20-39E1-4EAB-B87A-4809EC57D6A9}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{34ABFB4C-B909-4BAD-BD6D-1709B4BFF71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{283519F1-5C17-482F-8A34-D99A86FA489D}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19095" windowHeight="12075" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="303">
   <si>
     <t>FRENCH PPA MODEL — scenario_defaults.xlsx</t>
   </si>
@@ -1164,13 +1164,10 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1178,6 +1175,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
@@ -1195,6 +1195,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1491,7 +1495,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="17"/>
@@ -1533,17 +1537,17 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="20"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="19"/>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
@@ -1604,17 +1608,17 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="20"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="19"/>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
@@ -1791,17 +1795,17 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="20"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="19"/>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
@@ -1862,17 +1866,17 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="20"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="19"/>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
@@ -1962,17 +1966,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="20"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="19"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
@@ -2091,17 +2095,17 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="21" t="s">
+      <c r="A25" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="20"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="19"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
@@ -2223,8 +2227,8 @@
       <c r="A30" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>37</v>
+      <c r="B30" s="4">
+        <v>10</v>
       </c>
       <c r="C30" s="4">
         <v>10</v>
@@ -2307,17 +2311,17 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="21" t="s">
+      <c r="A33" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="20"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="19"/>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
@@ -2523,17 +2527,17 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="21" t="s">
+      <c r="A41" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="20"/>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="19"/>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
@@ -2768,17 +2772,17 @@
       </c>
     </row>
     <row r="50" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="21" t="s">
+      <c r="A50" s="20" t="s">
         <v>128</v>
       </c>
-      <c r="B50" s="19"/>
-      <c r="C50" s="19"/>
-      <c r="D50" s="19"/>
-      <c r="E50" s="19"/>
-      <c r="F50" s="19"/>
-      <c r="G50" s="19"/>
-      <c r="H50" s="19"/>
-      <c r="I50" s="20"/>
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="19"/>
     </row>
     <row r="51" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
@@ -2984,30 +2988,30 @@
       </c>
     </row>
     <row r="58" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="21" t="s">
+      <c r="A58" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="B58" s="19"/>
-      <c r="C58" s="19"/>
-      <c r="D58" s="19"/>
-      <c r="E58" s="19"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="19"/>
-      <c r="I58" s="20"/>
+      <c r="B58" s="18"/>
+      <c r="C58" s="18"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18"/>
+      <c r="I58" s="19"/>
     </row>
     <row r="59" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="B59" s="19"/>
-      <c r="C59" s="19"/>
-      <c r="D59" s="19"/>
-      <c r="E59" s="19"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="19"/>
-      <c r="I59" s="20"/>
+      <c r="B59" s="18"/>
+      <c r="C59" s="18"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="18"/>
+      <c r="F59" s="18"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="18"/>
+      <c r="I59" s="19"/>
     </row>
     <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
@@ -3068,30 +3072,30 @@
       </c>
     </row>
     <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A62" s="22" t="s">
+      <c r="A62" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B62" s="19"/>
-      <c r="C62" s="19"/>
-      <c r="D62" s="19"/>
-      <c r="E62" s="19"/>
-      <c r="F62" s="19"/>
-      <c r="G62" s="19"/>
-      <c r="H62" s="19"/>
-      <c r="I62" s="20"/>
+      <c r="B62" s="18"/>
+      <c r="C62" s="18"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="18"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="18"/>
+      <c r="I62" s="19"/>
     </row>
     <row r="63" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A63" s="18" t="s">
+      <c r="A63" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B63" s="19"/>
-      <c r="C63" s="19"/>
-      <c r="D63" s="19"/>
-      <c r="E63" s="19"/>
-      <c r="F63" s="19"/>
-      <c r="G63" s="19"/>
-      <c r="H63" s="19"/>
-      <c r="I63" s="20"/>
+      <c r="B63" s="18"/>
+      <c r="C63" s="18"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="18"/>
+      <c r="F63" s="18"/>
+      <c r="G63" s="18"/>
+      <c r="H63" s="18"/>
+      <c r="I63" s="19"/>
     </row>
     <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
@@ -3152,17 +3156,17 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="19"/>
-      <c r="C66" s="19"/>
-      <c r="D66" s="19"/>
-      <c r="E66" s="19"/>
-      <c r="F66" s="19"/>
-      <c r="G66" s="19"/>
-      <c r="H66" s="19"/>
-      <c r="I66" s="20"/>
+      <c r="B66" s="18"/>
+      <c r="C66" s="18"/>
+      <c r="D66" s="18"/>
+      <c r="E66" s="18"/>
+      <c r="F66" s="18"/>
+      <c r="G66" s="18"/>
+      <c r="H66" s="18"/>
+      <c r="I66" s="19"/>
     </row>
     <row r="67" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
@@ -3252,17 +3256,17 @@
       </c>
     </row>
     <row r="70" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A70" s="18" t="s">
+      <c r="A70" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="B70" s="19"/>
-      <c r="C70" s="19"/>
-      <c r="D70" s="19"/>
-      <c r="E70" s="19"/>
-      <c r="F70" s="19"/>
-      <c r="G70" s="19"/>
-      <c r="H70" s="19"/>
-      <c r="I70" s="20"/>
+      <c r="B70" s="18"/>
+      <c r="C70" s="18"/>
+      <c r="D70" s="18"/>
+      <c r="E70" s="18"/>
+      <c r="F70" s="18"/>
+      <c r="G70" s="18"/>
+      <c r="H70" s="18"/>
+      <c r="I70" s="19"/>
     </row>
     <row r="71" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="3" t="s">
@@ -3352,17 +3356,17 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A74" s="18" t="s">
+      <c r="A74" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="B74" s="19"/>
-      <c r="C74" s="19"/>
-      <c r="D74" s="19"/>
-      <c r="E74" s="19"/>
-      <c r="F74" s="19"/>
-      <c r="G74" s="19"/>
-      <c r="H74" s="19"/>
-      <c r="I74" s="20"/>
+      <c r="B74" s="18"/>
+      <c r="C74" s="18"/>
+      <c r="D74" s="18"/>
+      <c r="E74" s="18"/>
+      <c r="F74" s="18"/>
+      <c r="G74" s="18"/>
+      <c r="H74" s="18"/>
+      <c r="I74" s="19"/>
     </row>
     <row r="75" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="3" t="s">
@@ -3452,7 +3456,7 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" s="21" t="s">
+      <c r="A78" s="20" t="s">
         <v>183</v>
       </c>
       <c r="B78" s="17"/>
@@ -3465,7 +3469,7 @@
       <c r="I78" s="17"/>
     </row>
     <row r="79" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="18" t="s">
+      <c r="A79" s="16" t="s">
         <v>184</v>
       </c>
       <c r="B79" s="17"/>
@@ -3681,7 +3685,7 @@
       </c>
     </row>
     <row r="87" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" s="18" t="s">
+      <c r="A87" s="16" t="s">
         <v>203</v>
       </c>
       <c r="B87" s="17"/>
@@ -3868,7 +3872,7 @@
       </c>
     </row>
     <row r="94" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A94" s="18" t="s">
+      <c r="A94" s="16" t="s">
         <v>221</v>
       </c>
       <c r="B94" s="17"/>
@@ -4026,7 +4030,7 @@
       </c>
     </row>
     <row r="100" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A100" s="18" t="s">
+      <c r="A100" s="16" t="s">
         <v>234</v>
       </c>
       <c r="B100" s="17"/>
@@ -4325,7 +4329,7 @@
       <c r="H111" s="11"/>
       <c r="I111" s="12"/>
     </row>
-    <row r="112" spans="1:9" ht="34.9" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:9" ht="23.25" x14ac:dyDescent="0.45">
       <c r="A112" s="3" t="s">
         <v>262</v>
       </c>
@@ -4443,6 +4447,15 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A94:I94"/>
+    <mergeCell ref="A70:I70"/>
+    <mergeCell ref="A79:I79"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A87:I87"/>
+    <mergeCell ref="A78:I78"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A100:I100"/>
     <mergeCell ref="A63:I63"/>
     <mergeCell ref="A13:I13"/>
@@ -4456,15 +4469,6 @@
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A62:I62"/>
     <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A94:I94"/>
-    <mergeCell ref="A70:I70"/>
-    <mergeCell ref="A79:I79"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A87:I87"/>
-    <mergeCell ref="A78:I78"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update scenario_defaults.xlsx to reflect changes in data configurations
</commit_message>
<xml_diff>
--- a/database/scenario_defaults.xlsx
+++ b/database/scenario_defaults.xlsx
@@ -1164,10 +1164,13 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1175,9 +1178,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
@@ -1495,7 +1495,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="28.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="17"/>
@@ -1537,17 +1537,17 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="20"/>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
@@ -1608,17 +1608,17 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="20"/>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
@@ -1795,17 +1795,17 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="19"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="20"/>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
@@ -1866,17 +1866,17 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="19"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="20"/>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
@@ -1966,17 +1966,17 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="19"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
@@ -2095,17 +2095,17 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A25" s="20" t="s">
+      <c r="A25" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="19"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="20"/>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
@@ -2311,17 +2311,17 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B33" s="18"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="18"/>
-      <c r="I33" s="19"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="20"/>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="3" t="s">
@@ -2527,17 +2527,17 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A41" s="20" t="s">
+      <c r="A41" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="18"/>
-      <c r="G41" s="18"/>
-      <c r="H41" s="18"/>
-      <c r="I41" s="19"/>
+      <c r="B41" s="19"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="19"/>
+      <c r="H41" s="19"/>
+      <c r="I41" s="20"/>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="3" t="s">
@@ -2772,17 +2772,17 @@
       </c>
     </row>
     <row r="50" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="20" t="s">
+      <c r="A50" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B50" s="18"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="18"/>
-      <c r="F50" s="18"/>
-      <c r="G50" s="18"/>
-      <c r="H50" s="18"/>
-      <c r="I50" s="19"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
+      <c r="E50" s="19"/>
+      <c r="F50" s="19"/>
+      <c r="G50" s="19"/>
+      <c r="H50" s="19"/>
+      <c r="I50" s="20"/>
     </row>
     <row r="51" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="3" t="s">
@@ -2988,30 +2988,30 @@
       </c>
     </row>
     <row r="58" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A58" s="20" t="s">
+      <c r="A58" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B58" s="18"/>
-      <c r="C58" s="18"/>
-      <c r="D58" s="18"/>
-      <c r="E58" s="18"/>
-      <c r="F58" s="18"/>
-      <c r="G58" s="18"/>
-      <c r="H58" s="18"/>
-      <c r="I58" s="19"/>
+      <c r="B58" s="19"/>
+      <c r="C58" s="19"/>
+      <c r="D58" s="19"/>
+      <c r="E58" s="19"/>
+      <c r="F58" s="19"/>
+      <c r="G58" s="19"/>
+      <c r="H58" s="19"/>
+      <c r="I58" s="20"/>
     </row>
     <row r="59" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A59" s="16" t="s">
+      <c r="A59" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="B59" s="18"/>
-      <c r="C59" s="18"/>
-      <c r="D59" s="18"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="18"/>
-      <c r="G59" s="18"/>
-      <c r="H59" s="18"/>
-      <c r="I59" s="19"/>
+      <c r="B59" s="19"/>
+      <c r="C59" s="19"/>
+      <c r="D59" s="19"/>
+      <c r="E59" s="19"/>
+      <c r="F59" s="19"/>
+      <c r="G59" s="19"/>
+      <c r="H59" s="19"/>
+      <c r="I59" s="20"/>
     </row>
     <row r="60" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="3" t="s">
@@ -3072,30 +3072,30 @@
       </c>
     </row>
     <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A62" s="21" t="s">
+      <c r="A62" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="B62" s="18"/>
-      <c r="C62" s="18"/>
-      <c r="D62" s="18"/>
-      <c r="E62" s="18"/>
-      <c r="F62" s="18"/>
-      <c r="G62" s="18"/>
-      <c r="H62" s="18"/>
-      <c r="I62" s="19"/>
+      <c r="B62" s="19"/>
+      <c r="C62" s="19"/>
+      <c r="D62" s="19"/>
+      <c r="E62" s="19"/>
+      <c r="F62" s="19"/>
+      <c r="G62" s="19"/>
+      <c r="H62" s="19"/>
+      <c r="I62" s="20"/>
     </row>
     <row r="63" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A63" s="16" t="s">
+      <c r="A63" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="B63" s="18"/>
-      <c r="C63" s="18"/>
-      <c r="D63" s="18"/>
-      <c r="E63" s="18"/>
-      <c r="F63" s="18"/>
-      <c r="G63" s="18"/>
-      <c r="H63" s="18"/>
-      <c r="I63" s="19"/>
+      <c r="B63" s="19"/>
+      <c r="C63" s="19"/>
+      <c r="D63" s="19"/>
+      <c r="E63" s="19"/>
+      <c r="F63" s="19"/>
+      <c r="G63" s="19"/>
+      <c r="H63" s="19"/>
+      <c r="I63" s="20"/>
     </row>
     <row r="64" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="3" t="s">
@@ -3156,17 +3156,17 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A66" s="16" t="s">
+      <c r="A66" s="18" t="s">
         <v>155</v>
       </c>
-      <c r="B66" s="18"/>
-      <c r="C66" s="18"/>
-      <c r="D66" s="18"/>
-      <c r="E66" s="18"/>
-      <c r="F66" s="18"/>
-      <c r="G66" s="18"/>
-      <c r="H66" s="18"/>
-      <c r="I66" s="19"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="19"/>
+      <c r="D66" s="19"/>
+      <c r="E66" s="19"/>
+      <c r="F66" s="19"/>
+      <c r="G66" s="19"/>
+      <c r="H66" s="19"/>
+      <c r="I66" s="20"/>
     </row>
     <row r="67" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="3" t="s">
@@ -3256,17 +3256,17 @@
       </c>
     </row>
     <row r="70" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A70" s="16" t="s">
+      <c r="A70" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="B70" s="18"/>
-      <c r="C70" s="18"/>
-      <c r="D70" s="18"/>
-      <c r="E70" s="18"/>
-      <c r="F70" s="18"/>
-      <c r="G70" s="18"/>
-      <c r="H70" s="18"/>
-      <c r="I70" s="19"/>
+      <c r="B70" s="19"/>
+      <c r="C70" s="19"/>
+      <c r="D70" s="19"/>
+      <c r="E70" s="19"/>
+      <c r="F70" s="19"/>
+      <c r="G70" s="19"/>
+      <c r="H70" s="19"/>
+      <c r="I70" s="20"/>
     </row>
     <row r="71" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="3" t="s">
@@ -3356,17 +3356,17 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A74" s="16" t="s">
+      <c r="A74" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="B74" s="18"/>
-      <c r="C74" s="18"/>
-      <c r="D74" s="18"/>
-      <c r="E74" s="18"/>
-      <c r="F74" s="18"/>
-      <c r="G74" s="18"/>
-      <c r="H74" s="18"/>
-      <c r="I74" s="19"/>
+      <c r="B74" s="19"/>
+      <c r="C74" s="19"/>
+      <c r="D74" s="19"/>
+      <c r="E74" s="19"/>
+      <c r="F74" s="19"/>
+      <c r="G74" s="19"/>
+      <c r="H74" s="19"/>
+      <c r="I74" s="20"/>
     </row>
     <row r="75" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="3" t="s">
@@ -3456,7 +3456,7 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A78" s="20" t="s">
+      <c r="A78" s="21" t="s">
         <v>183</v>
       </c>
       <c r="B78" s="17"/>
@@ -3469,7 +3469,7 @@
       <c r="I78" s="17"/>
     </row>
     <row r="79" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A79" s="16" t="s">
+      <c r="A79" s="18" t="s">
         <v>184</v>
       </c>
       <c r="B79" s="17"/>
@@ -3685,7 +3685,7 @@
       </c>
     </row>
     <row r="87" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A87" s="16" t="s">
+      <c r="A87" s="18" t="s">
         <v>203</v>
       </c>
       <c r="B87" s="17"/>
@@ -3872,7 +3872,7 @@
       </c>
     </row>
     <row r="94" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A94" s="16" t="s">
+      <c r="A94" s="18" t="s">
         <v>221</v>
       </c>
       <c r="B94" s="17"/>
@@ -4030,7 +4030,7 @@
       </c>
     </row>
     <row r="100" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A100" s="16" t="s">
+      <c r="A100" s="18" t="s">
         <v>234</v>
       </c>
       <c r="B100" s="17"/>
@@ -4447,15 +4447,6 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A94:I94"/>
-    <mergeCell ref="A70:I70"/>
-    <mergeCell ref="A79:I79"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="A87:I87"/>
-    <mergeCell ref="A78:I78"/>
-    <mergeCell ref="A16:I16"/>
-    <mergeCell ref="A3:I3"/>
     <mergeCell ref="A100:I100"/>
     <mergeCell ref="A63:I63"/>
     <mergeCell ref="A13:I13"/>
@@ -4469,6 +4460,15 @@
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A62:I62"/>
     <mergeCell ref="A20:I20"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A94:I94"/>
+    <mergeCell ref="A70:I70"/>
+    <mergeCell ref="A79:I79"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A87:I87"/>
+    <mergeCell ref="A78:I78"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>